<commit_message>
bench: links written, Excel's answers on the Mac after the rich values
The writer stored #SPILL! and #CALC! of a link as #VALUE! with their rich values:
Excel for Mac opened all seven files and showed #VALUE! for both (ERROR.TYPE 3),
the alternative the case errors gave, and saved them as plain #VALUE! without
the rich values. The other six cases answered as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/links/written/cache.xlsx
+++ b/test/excel/links/written/cache.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-23390/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-39313/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FC8C534-5CF4-0A4C-B7B6-BABFA49DBAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{979ADDCE-D5B8-7842-8236-44D2EB3AE2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
bench: links written, Excel's answers on the Mac with plain #VALUE!
All seven files open; 72 of the 76 predicted values as predicted, the four of the
case errors as its alternative (#SPILL! and #CALC! of a link show #VALUE!).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/links/written/cache.xlsx
+++ b/test/excel/links/written/cache.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-39313/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-51168/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{979ADDCE-D5B8-7842-8236-44D2EB3AE2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E601A64-6A13-9243-A8A0-C02B37813E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>